<commit_message>
feat(seago): enhance PO Excel import/export with validation and fix color normalization
- Add color normalization in StylesPart to properly format RGB colors
- Extend PropInfo schema with validation attributes (mandatory, pattern, min/max, precision, scale, minLength, maxLength)
- Add parseExcel method for reading Excel files into PO models
- Simplify export workflow by removing complex dict/list options handling
- Add dictionary label conversion during export
- Update tests with new validation and parsing scenarios
</commit_message>
<xml_diff>
--- a/nop-seago/nop-seago-list/src/test/resources/_vfs/seago/po/test.xlsx
+++ b/nop-seago/nop-seago-list/src/test/resources/_vfs/seago/po/test.xlsx
@@ -43,9 +43,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="2">
     <font>
-      <name/>
+      <name val="Calibri"/>
+      <sz val="11"/>
+      <family val="2"/>
+      <color rgb="0"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b/>
     </font>
   </fonts>
@@ -58,38 +64,47 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="C0C0C0"/>
+        <fgColor rgb="FFC0C0C0"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
-      <left style="thin">
-        <color rgb="000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="000000"/>
-      </bottom>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="000000"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="000000"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color rgb="000000"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="000000"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -98,10 +113,10 @@
     </xf>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf fontId="0" fillId="2" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0">
       <alignment vertical="center" horizontal="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -414,7 +429,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -458,6 +473,24 @@
         </is>
       </c>
       <c r="D3" s="0"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>1001</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>ZhangSan</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>男</t>
+        </is>
+      </c>
+      <c r="D4" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -466,13 +499,5 @@
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:D3"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4:C1048576">
-      <formula1>""</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4:D1048576">
-      <formula1>""</formula1>
-    </dataValidation>
-  </dataValidations>
 </worksheet>
 </file>
</xml_diff>